<commit_message>
new treasury features v2
</commit_message>
<xml_diff>
--- a/public/BA_treasury_report.xlsx
+++ b/public/BA_treasury_report.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E14"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -424,10 +424,10 @@
         <v>Credit</v>
       </c>
       <c r="C2">
-        <v>1229</v>
+        <v>34</v>
       </c>
       <c r="D2" t="str">
-        <v>bowa</v>
+        <v>344</v>
       </c>
       <c r="E2" t="str">
         <v>BA</v>
@@ -586,9 +586,60 @@
         <v>Unknown</v>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>26/03/2026</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Credit</v>
+      </c>
+      <c r="C12">
+        <v>1229</v>
+      </c>
+      <c r="D12" t="str">
+        <v>bowa</v>
+      </c>
+      <c r="E12" t="str">
+        <v>Unknown</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>26/03/2026</v>
+      </c>
+      <c r="B13" t="str">
+        <v>Debit</v>
+      </c>
+      <c r="C13">
+        <v>223</v>
+      </c>
+      <c r="D13" t="str">
+        <v>ddz</v>
+      </c>
+      <c r="E13" t="str">
+        <v>Unknown</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>26/03/2026</v>
+      </c>
+      <c r="B14" t="str">
+        <v>Debit</v>
+      </c>
+      <c r="C14">
+        <v>23</v>
+      </c>
+      <c r="D14" t="str">
+        <v>dede</v>
+      </c>
+      <c r="E14" t="str">
+        <v>Unknown</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E14"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>